<commit_message>
Make MRP or LP a two-value selector instead of a currency amount
mrp_or_lp only ever holds "MRP" or "LP" -- changed from a numeric
field to a select everywhere it's edited (Item Master table, Create
Item dialog) and imported (.xlsx upload, Google Sheet sync), with a
DB check constraint enforcing the two allowed values.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012eh6G732LxQZxzYXJ63qeK
</commit_message>
<xml_diff>
--- a/public/templates/item-master-template.xlsx
+++ b/public/templates/item-master-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>sku</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>MRP</t>
   </si>
   <si>
     <t>85362090</t>
@@ -502,7 +505,8 @@
     <col min="13" max="14" width="12" customWidth="1"/>
     <col min="15" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="40" customWidth="1"/>
-    <col min="18" max="19" width="12" customWidth="1"/>
+    <col min="18" max="18" width="12" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
     <col min="20" max="20" width="14" customWidth="1"/>
     <col min="21" max="21" width="32" customWidth="1"/>
   </cols>
@@ -624,14 +628,14 @@
       <c r="R2" t="s">
         <v>30</v>
       </c>
-      <c r="S2">
-        <v>1250</v>
+      <c r="S2" t="s">
+        <v>31</v>
       </c>
       <c r="T2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="U2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>